<commit_message>
delete unnecessary files and change learn and retr generation files to always start a new block with the new image sequence
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/learning_block1_fixed-middle-10_02.xlsx
+++ b/psychopy_exp_files/sequences/learning_block1_fixed-middle-10_02.xlsx
@@ -604,17 +604,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S2" t="n">
@@ -703,7 +703,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P3" t="n">
@@ -724,7 +724,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S3" t="n">
@@ -802,7 +802,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P4" t="n">
@@ -823,7 +823,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S4" t="n">
@@ -906,12 +906,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -1000,17 +1000,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P6" t="n">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S6" t="n">
@@ -1099,17 +1099,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S7" t="n">
@@ -1168,12 +1168,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1188,38 +1188,38 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>key</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S8" t="n">
@@ -1232,10 +1232,10 @@
         <v>4</v>
       </c>
       <c r="V8" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="W8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1297,28 +1297,28 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="Q9" t="n">
         <v>0.2</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S9" t="n">
@@ -1331,7 +1331,7 @@
         <v>7</v>
       </c>
       <c r="V9" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="W9" t="n">
         <v>9</v>
@@ -1366,12 +1366,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1410,10 +1410,10 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.6</v>
+        <v>0.53</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.33</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1430,10 +1430,10 @@
         <v>6</v>
       </c>
       <c r="V10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1485,38 +1485,38 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.47</v>
+        <v>0.67</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.33</v>
+        <v>0.53</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S11" t="n">
@@ -1529,10 +1529,10 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="W11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1564,12 +1564,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1584,17 +1584,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1604,18 +1604,18 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S12" t="n">
@@ -1628,10 +1628,10 @@
         <v>2</v>
       </c>
       <c r="V12" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="W12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_26.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1683,38 +1683,38 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.53</v>
+        <v>0.73</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.27</v>
+        <v>0.47</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S13" t="n">
@@ -1727,10 +1727,10 @@
         <v>15</v>
       </c>
       <c r="V13" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="W13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -1762,12 +1762,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1782,38 +1782,38 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.8</v>
+        <v>0.67</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.47</v>
+        <v>0.33</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S14" t="n">
@@ -1826,10 +1826,10 @@
         <v>17</v>
       </c>
       <c r="V14" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="W14" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1891,28 +1891,28 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.64</v>
+        <v>0.75</v>
       </c>
       <c r="Q15" t="n">
         <v>0.36</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S15" t="n">
@@ -1925,7 +1925,7 @@
         <v>14</v>
       </c>
       <c r="V15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="W15" t="n">
         <v>1</v>
@@ -1960,12 +1960,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_26.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1980,22 +1980,22 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>key</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2004,14 +2004,14 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.53</v>
+        <v>0.31</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S16" t="n">
@@ -2024,10 +2024,10 @@
         <v>8</v>
       </c>
       <c r="V16" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="W16" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2079,17 +2079,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2099,18 +2099,18 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.42</v>
+        <v>0.58</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S17" t="n">
@@ -2123,10 +2123,10 @@
         <v>3</v>
       </c>
       <c r="V17" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W17" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2178,12 +2178,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2193,19 +2193,19 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.42</v>
+        <v>0.64</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -2222,10 +2222,10 @@
         <v>5</v>
       </c>
       <c r="V18" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="W18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -2292,12 +2292,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P19" t="n">
@@ -2356,12 +2356,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2376,38 +2376,38 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.47</v>
+        <v>0.33</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S20" t="n">
@@ -2420,10 +2420,10 @@
         <v>10</v>
       </c>
       <c r="V20" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="W20" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -2455,12 +2455,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2475,38 +2475,38 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.33</v>
+        <v>0.8</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.2</v>
+        <v>0.53</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S21" t="n">
@@ -2519,10 +2519,10 @@
         <v>4</v>
       </c>
       <c r="V21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W21" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2579,17 +2579,17 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -2601,11 +2601,11 @@
         <v>0.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.58</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S22" t="n">
@@ -2621,7 +2621,7 @@
         <v>6</v>
       </c>
       <c r="W22" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -2653,12 +2653,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2673,12 +2673,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>key</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2688,19 +2688,19 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -2717,10 +2717,10 @@
         <v>6</v>
       </c>
       <c r="V23" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="W23" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2792,18 +2792,18 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.33</v>
       </c>
       <c r="Q24" t="n">
         <v>0.2</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S24" t="n">
@@ -2816,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="V24" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="W24" t="n">
         <v>4</v>
@@ -2851,12 +2851,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2871,12 +2871,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2886,19 +2886,19 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.6</v>
+        <v>0.47</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -2915,10 +2915,10 @@
         <v>2</v>
       </c>
       <c r="V25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W25" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3079,28 +3079,28 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.47</v>
+        <v>0.6</v>
       </c>
       <c r="Q27" t="n">
         <v>0.27</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S27" t="n">
@@ -3113,7 +3113,7 @@
         <v>17</v>
       </c>
       <c r="V27" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W27" t="n">
         <v>6</v>
@@ -3148,12 +3148,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/flower/flower_22.jpg</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3168,17 +3168,17 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3188,18 +3188,18 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S28" t="n">
@@ -3212,10 +3212,10 @@
         <v>14</v>
       </c>
       <c r="V28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="W28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -3247,12 +3247,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_26.jpg</t>
+          <t>stimuli/chair/chair_16.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/ball/ball_23.jpg</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3267,22 +3267,22 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3291,14 +3291,14 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S29" t="n">
@@ -3311,10 +3311,10 @@
         <v>8</v>
       </c>
       <c r="V29" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="W29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -3346,12 +3346,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_22.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3366,12 +3366,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>key</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3390,10 +3390,10 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.75</v>
+        <v>0.58</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.53</v>
+        <v>0.36</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -3410,10 +3410,10 @@
         <v>3</v>
       </c>
       <c r="V30" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W30" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -3475,17 +3475,17 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P31" t="n">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S31" t="n">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_22.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3574,12 +3574,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -3588,14 +3588,14 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.64</v>
+        <v>0.53</v>
       </c>
       <c r="Q32" t="n">
         <v>0.42</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S32" t="n">
@@ -3608,7 +3608,7 @@
         <v>9</v>
       </c>
       <c r="V32" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W32" t="n">
         <v>17</v>
@@ -3643,14 +3643,14 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>stimuli/key/key_39.jpg</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>stimuli/hand/hand_30.jpg</t>
-        </is>
-      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>house</t>
@@ -3663,14 +3663,14 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
           <t>guitar</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>hand</t>
-        </is>
-      </c>
       <c r="M33" t="inlineStr">
         <is>
           <t>center</t>
@@ -3678,19 +3678,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P33" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="Q33" t="n">
         <v>0.4</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>0.27</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -3707,10 +3707,10 @@
         <v>10</v>
       </c>
       <c r="V33" t="n">
+        <v>15</v>
+      </c>
+      <c r="W33" t="n">
         <v>13</v>
-      </c>
-      <c r="W33" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="34">
@@ -3742,12 +3742,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3762,38 +3762,38 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.47</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.58</v>
+        <v>0.33</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S34" t="n">
@@ -3806,10 +3806,10 @@
         <v>4</v>
       </c>
       <c r="V34" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="W34" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3866,12 +3866,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P35" t="n">
         <v>0.47</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S35" t="n">
@@ -3908,7 +3908,7 @@
         <v>14</v>
       </c>
       <c r="W35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3960,38 +3960,38 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S36" t="n">
@@ -4004,10 +4004,10 @@
         <v>6</v>
       </c>
       <c r="V36" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -4083,7 +4083,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="Q37" t="n">
         <v>0.2</v>
@@ -4103,7 +4103,7 @@
         <v>1</v>
       </c>
       <c r="V37" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="W37" t="n">
         <v>4</v>
@@ -4138,12 +4138,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4158,38 +4158,38 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.53</v>
+        <v>0.33</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S38" t="n">
@@ -4202,10 +4202,10 @@
         <v>2</v>
       </c>
       <c r="V38" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="W38" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4257,12 +4257,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4281,10 +4281,10 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.47</v>
+        <v>0.27</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -4301,10 +4301,10 @@
         <v>15</v>
       </c>
       <c r="V39" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="W39" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4376,18 +4376,18 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.8</v>
+        <v>0.73</v>
       </c>
       <c r="Q40" t="n">
         <v>0.4</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S40" t="n">
@@ -4400,7 +4400,7 @@
         <v>17</v>
       </c>
       <c r="V40" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="W40" t="n">
         <v>4</v>
@@ -4435,12 +4435,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/ball/ball_23.jpg</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4455,38 +4455,38 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S41" t="n">
@@ -4499,10 +4499,10 @@
         <v>14</v>
       </c>
       <c r="V41" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -4534,12 +4534,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_22.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4554,22 +4554,22 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -4578,14 +4578,14 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.64</v>
+        <v>0.53</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.47</v>
+        <v>0.36</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S42" t="n">
@@ -4598,10 +4598,10 @@
         <v>8</v>
       </c>
       <c r="V42" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="W42" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -4633,12 +4633,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_26.jpg</t>
+          <t>stimuli/ball/ball_23.jpg</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4653,38 +4653,38 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.58</v>
+        <v>0.47</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S43" t="n">
@@ -4697,10 +4697,10 @@
         <v>3</v>
       </c>
       <c r="V43" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="W43" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_22.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -4776,10 +4776,10 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.58</v>
+        <v>0.64</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -4796,10 +4796,10 @@
         <v>5</v>
       </c>
       <c r="V44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W44" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/chair/chair_16.jpg</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4851,38 +4851,38 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.42</v>
+        <v>0.53</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S45" t="n">
@@ -4895,10 +4895,10 @@
         <v>9</v>
       </c>
       <c r="V45" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="W45" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -4930,12 +4930,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_26.jpg</t>
+          <t>stimuli/flower/flower_22.jpg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4950,17 +4950,17 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>key</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -4970,18 +4970,18 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.75</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.64</v>
+        <v>0.53</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S46" t="n">
@@ -4994,10 +4994,10 @@
         <v>10</v>
       </c>
       <c r="V46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W46" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47">
@@ -5029,12 +5029,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5049,17 +5049,17 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5069,18 +5069,18 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.47</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.47</v>
+        <v>0.27</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S47" t="n">
@@ -5093,10 +5093,10 @@
         <v>4</v>
       </c>
       <c r="V47" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="W47" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -5128,12 +5128,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5148,12 +5148,12 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5172,10 +5172,10 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.64</v>
+        <v>0.47</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -5192,10 +5192,10 @@
         <v>7</v>
       </c>
       <c r="V48" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49">
@@ -5227,12 +5227,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5247,12 +5247,12 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -5271,10 +5271,10 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>0.53</v>
+        <v>0.47</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -5291,10 +5291,10 @@
         <v>6</v>
       </c>
       <c r="V49" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="W49" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -5326,12 +5326,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5346,38 +5346,38 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.33</v>
+        <v>0.8</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.2</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S50" t="n">
@@ -5390,10 +5390,10 @@
         <v>1</v>
       </c>
       <c r="V50" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="W50" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="51">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -5460,19 +5460,19 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P51" t="n">
         <v>0.6</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
@@ -5492,7 +5492,7 @@
         <v>8</v>
       </c>
       <c r="W51" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -5559,16 +5559,16 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>0.6</v>
+        <v>0.53</v>
       </c>
       <c r="Q52" t="n">
         <v>0.27</v>
@@ -5588,7 +5588,7 @@
         <v>15</v>
       </c>
       <c r="V52" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W52" t="n">
         <v>7</v>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -5653,12 +5653,12 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -5667,14 +5667,14 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>0.73</v>
+        <v>0.8</v>
       </c>
       <c r="Q53" t="n">
         <v>0.4</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S53" t="n">
@@ -5687,7 +5687,7 @@
         <v>17</v>
       </c>
       <c r="V53" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="W53" t="n">
         <v>4</v>
@@ -5722,12 +5722,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5742,38 +5742,38 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>0.8</v>
+        <v>0.64</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S54" t="n">
@@ -5786,10 +5786,10 @@
         <v>14</v>
       </c>
       <c r="V54" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -5821,12 +5821,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5841,17 +5841,17 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>key</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -5861,18 +5861,18 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P55" t="n">
-        <v>0.58</v>
+        <v>0.75</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S55" t="n">
@@ -5885,10 +5885,10 @@
         <v>8</v>
       </c>
       <c r="V55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W55" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56">
@@ -5950,12 +5950,12 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S56" t="n">
@@ -6019,12 +6019,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6039,38 +6039,38 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>0.53</v>
+        <v>0.75</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.42</v>
+        <v>0.64</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S57" t="n">
@@ -6083,10 +6083,10 @@
         <v>5</v>
       </c>
       <c r="V57" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="W57" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/ball/ball_23.jpg</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -6165,7 +6165,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
@@ -6185,7 +6185,7 @@
         <v>7</v>
       </c>
       <c r="W58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/chair/chair_16.jpg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6237,17 +6237,17 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>key</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -6257,18 +6257,18 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P59" t="n">
-        <v>0.58</v>
+        <v>0.8</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.4</v>
+        <v>0.53</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S59" t="n">
@@ -6281,10 +6281,10 @@
         <v>10</v>
       </c>
       <c r="V59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W59" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60">
@@ -6316,7 +6316,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -6346,28 +6346,28 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="Q60" t="n">
         <v>0.2</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S60" t="n">
@@ -6380,7 +6380,7 @@
         <v>4</v>
       </c>
       <c r="V60" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="W60" t="n">
         <v>5</v>
@@ -6415,14 +6415,14 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
+          <t>stimuli/key/key_39.jpg</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
           <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>stimuli/house/house_05.jpg</t>
-        </is>
-      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>chair</t>
@@ -6435,38 +6435,38 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
           <t>guitar</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>house</t>
-        </is>
-      </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P61" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="Q61" t="n">
         <v>0.53</v>
       </c>
-      <c r="Q61" t="n">
-        <v>0.2</v>
-      </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S61" t="n">
@@ -6479,10 +6479,10 @@
         <v>7</v>
       </c>
       <c r="V61" t="n">
+        <v>15</v>
+      </c>
+      <c r="W61" t="n">
         <v>13</v>
-      </c>
-      <c r="W61" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="62">
@@ -6514,12 +6514,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6534,38 +6534,38 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P62" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.4</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S62" t="n">
@@ -6578,10 +6578,10 @@
         <v>6</v>
       </c>
       <c r="V62" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="W62" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63">
@@ -6613,12 +6613,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6633,38 +6633,38 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P63" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q63" t="n">
-        <v>0.27</v>
+        <v>0.47</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S63" t="n">
@@ -6677,10 +6677,10 @@
         <v>1</v>
       </c>
       <c r="V63" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="W63" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -6737,12 +6737,12 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -6752,18 +6752,18 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P64" t="n">
         <v>0.73</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.47</v>
+        <v>0.33</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S64" t="n">
@@ -6779,7 +6779,7 @@
         <v>13</v>
       </c>
       <c r="W64" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65">
@@ -6816,7 +6816,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/house/house_05.jpg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6836,7 +6836,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -6846,19 +6846,19 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P65" t="n">
         <v>0.67</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.33</v>
+        <v>0.47</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -6878,7 +6878,7 @@
         <v>8</v>
       </c>
       <c r="W65" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66">
@@ -6940,12 +6940,12 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S66" t="n">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>stimuli/house/house_05.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/flower/flower_22.jpg</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -7029,17 +7029,17 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -7049,18 +7049,18 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>0.64</v>
+        <v>0.8</v>
       </c>
       <c r="Q67" t="n">
-        <v>0.31</v>
+        <v>0.42</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S67" t="n">
@@ -7073,10 +7073,10 @@
         <v>14</v>
       </c>
       <c r="V67" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W67" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68">
@@ -7108,12 +7108,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_22.jpg</t>
+          <t>stimuli/hammer/hammer_26.jpg</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>stimuli/key/key_39.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7128,22 +7128,22 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -7152,14 +7152,14 @@
         </is>
       </c>
       <c r="P68" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.31</v>
+        <v>0.25</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S68" t="n">
@@ -7172,10 +7172,10 @@
         <v>8</v>
       </c>
       <c r="V68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W68" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="69">
@@ -7207,12 +7207,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/bicycle/bicycle_35.jpg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7227,38 +7227,38 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P69" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.31</v>
+        <v>0.42</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S69" t="n">
@@ -7271,10 +7271,10 @@
         <v>3</v>
       </c>
       <c r="V69" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W69" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
@@ -7306,12 +7306,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_35.jpg</t>
+          <t>stimuli/chair/chair_16.jpg</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_23.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7326,17 +7326,17 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -7346,18 +7346,18 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P70" t="n">
-        <v>0.75</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.53</v>
+        <v>0.36</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S70" t="n">
@@ -7370,10 +7370,10 @@
         <v>5</v>
       </c>
       <c r="V70" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="W70" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71">
@@ -7405,7 +7405,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/jacket/jacket_35.jpg</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -7425,7 +7425,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -7440,16 +7440,16 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P71" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="Q71" t="n">
         <v>0.27</v>
@@ -7469,7 +7469,7 @@
         <v>9</v>
       </c>
       <c r="V71" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="W71" t="n">
         <v>14</v>
@@ -7504,12 +7504,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_26.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7524,38 +7524,38 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P72" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="Q72" t="n">
-        <v>0.47</v>
+        <v>0.27</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S72" t="n">
@@ -7568,10 +7568,10 @@
         <v>10</v>
       </c>
       <c r="V72" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="W72" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="73">
@@ -7603,12 +7603,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/flower/flower_22.jpg</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_30.jpg</t>
+          <t>stimuli/key/key_39.jpg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7623,12 +7623,12 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>key</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -7647,10 +7647,10 @@
         </is>
       </c>
       <c r="P73" t="n">
-        <v>0.33</v>
+        <v>0.75</v>
       </c>
       <c r="Q73" t="n">
-        <v>0.2</v>
+        <v>0.58</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -7667,10 +7667,10 @@
         <v>4</v>
       </c>
       <c r="V73" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W73" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="74">
@@ -7702,12 +7702,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/guitar/guitar_13.jpg</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_49.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7722,38 +7722,38 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P74" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="Q74" t="n">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S74" t="n">
@@ -7766,10 +7766,10 @@
         <v>7</v>
       </c>
       <c r="V74" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="W74" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>0.6</v>
+        <v>0.53</v>
       </c>
       <c r="Q75" t="n">
         <v>0.27</v>
@@ -7865,7 +7865,7 @@
         <v>6</v>
       </c>
       <c r="V75" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W75" t="n">
         <v>9</v>
@@ -7900,12 +7900,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_35.jpg</t>
+          <t>stimuli/phone/phone_17.jpg</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>stimuli/phone/phone_17.jpg</t>
+          <t>stimuli/bread/bread_49.jpg</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7920,12 +7920,12 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -7944,10 +7944,10 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.47</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -7964,10 +7964,10 @@
         <v>1</v>
       </c>
       <c r="V76" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="W76" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
@@ -7999,7 +7999,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_30.jpg</t>
+          <t>stimuli/lamp/lamp_23.jpg</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -8019,7 +8019,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -8043,7 +8043,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>0.6</v>
+        <v>0.67</v>
       </c>
       <c r="Q77" t="n">
         <v>0.4</v>
@@ -8063,7 +8063,7 @@
         <v>2</v>
       </c>
       <c r="V77" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="W77" t="n">
         <v>9</v>
@@ -8098,12 +8098,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_23.jpg</t>
+          <t>stimuli/hand/hand_30.jpg</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/flower/flower_22.jpg</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -8118,22 +8118,22 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -8142,14 +8142,14 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>0.73</v>
+        <v>0.67</v>
       </c>
       <c r="Q78" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S78" t="n">
@@ -8162,10 +8162,10 @@
         <v>15</v>
       </c>
       <c r="V78" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="W78" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79">
@@ -8197,12 +8197,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_16.jpg</t>
+          <t>stimuli/dog/dog_30.jpg</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_13.jpg</t>
+          <t>stimuli/ball/ball_23.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -8217,12 +8217,12 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -8241,10 +8241,10 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -8261,10 +8261,10 @@
         <v>17</v>
       </c>
       <c r="V79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W79" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>